<commit_message>
Geokodowanie GUGiK, grupowanie wg stref trafo/miejscowości, pismo docx, zestawienia xlsx/xls, słowniki operatorów i rejonów
</commit_message>
<xml_diff>
--- a/dane/slowniki.xlsx
+++ b/dane/slowniki.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Operatorzy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Rejony" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operatorzy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejony" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,13 +26,21 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -47,8 +55,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,75 +423,113 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Nazwa</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Numer Umowy Ramowej</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Pełna nazwa</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Adres</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Adres (siedziba)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Kod pocztowy</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>NIP</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Osoba kontaktowa</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>E-mail</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Telefon</t>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Regon</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Numer wpisu do RPT</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Dane kontaktowe</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Operator A</t>
+          <t>InterWan</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Operator A Sp. z o.o.</t>
+          <t>1441OW2018</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ul. Przykładowa 1, 00-001 Warszawa</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+          <t>InterWan Sp z.o.o.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ul. Lazurowa 1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>05-331 Dębę Wielkie</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>8222349374</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>361015909</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>5522</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Marcin Macko tel. 502 761 590 marcin.macko@mmui.pl</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -495,68 +542,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Nazwa</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Oddział</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Adres</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Osoba kontaktowa</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>E-mail</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Telefon</t>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Gminy</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Uwagi</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rejon Energetyczny X</t>
+          <t>Rejon Energetyczny Mińsk Mazowiecki</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Oddział Y</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>ul. Przykładowa 2, 00-002 Miasto</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+          <t>Mińsk Mazowiecki; Mińsk Mazowiecki (miasto)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Okno programu (Qt), numeracja odnośnikami jak w numeracja_leader.dxf, scalanie błędnych klików do 5 m, strefy trafo z multileaderów, zestawienia wg szablonów
</commit_message>
<xml_diff>
--- a/dane/slowniki.xlsx
+++ b/dane/slowniki.xlsx
@@ -542,12 +542,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -558,10 +559,15 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Nazwa skrócona</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Gminy</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Uwagi</t>
         </is>
@@ -575,10 +581,33 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mińsk Mazowiecki; Mińsk Mazowiecki (miasto)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>Mińsk Mazowiecki</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Mińsk Mazowiecki; Mińsk Mazowiecki (miasto); Dębe Wielkie; Jakubów</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Rejon Energetyczny Otwock</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>OTWOCK</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Otwock; Józefów; Karczew; Celestynów; Halinów</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>